<commit_message>
Rohini: CreateUserCredentials - TestData
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -1,21 +1,71 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateUserCredentials" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Employeename</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>ConfirmPassword</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>ESS</t>
+  </si>
+  <si>
+    <t>Admin 1</t>
+  </si>
+  <si>
+    <t>Employee 1</t>
+  </si>
+  <si>
+    <t>Enabled</t>
+  </si>
+  <si>
+    <t>Admin_1</t>
+  </si>
+  <si>
+    <t>Employee_1</t>
+  </si>
+  <si>
+    <t>Admin123</t>
+  </si>
+  <si>
+    <t>Employee123</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,6 +102,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -98,7 +156,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -133,7 +191,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -341,10 +399,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rohini: Create User Credentials
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -49,16 +49,16 @@
     <t>Enabled</t>
   </si>
   <si>
-    <t>Admin_1</t>
-  </si>
-  <si>
-    <t>Employee_1</t>
-  </si>
-  <si>
     <t>Admin123</t>
   </si>
   <si>
     <t>Employee123</t>
+  </si>
+  <si>
+    <t>Admin_123</t>
+  </si>
+  <si>
+    <t>Employee_123</t>
   </si>
 </sst>
 </file>
@@ -434,13 +434,13 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -454,13 +454,13 @@
         <v>10</v>
       </c>
       <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rohini: Create User Credentials - Created Admin Credentials
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t>Role</t>
   </si>
@@ -55,10 +55,22 @@
     <t>Employee123</t>
   </si>
   <si>
-    <t>Admin@123</t>
-  </si>
-  <si>
-    <t>Employee@123</t>
+    <t>Admin 2</t>
+  </si>
+  <si>
+    <t>Admin2@123</t>
+  </si>
+  <si>
+    <t>Employee1@123</t>
+  </si>
+  <si>
+    <t>Admin1@123</t>
+  </si>
+  <si>
+    <t>Employee 2</t>
+  </si>
+  <si>
+    <t>Employee2@123</t>
   </si>
 </sst>
 </file>
@@ -411,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -445,7 +457,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
@@ -465,12 +477,52 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
       </c>
       <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
         <v>12</v>
       </c>
     </row>
@@ -478,6 +530,8 @@
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1"/>
     <hyperlink ref="D3" r:id="rId2"/>
+    <hyperlink ref="D4" r:id="rId3"/>
+    <hyperlink ref="D5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Rohini: Create User Credentials - Updated Employee Credentials
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
   <si>
     <t>Role</t>
   </si>
@@ -71,6 +71,12 @@
   </si>
   <si>
     <t>Employee2@123</t>
+  </si>
+  <si>
+    <t>UserFilter</t>
+  </si>
+  <si>
+    <t>Employee</t>
   </si>
 </sst>
 </file>
@@ -423,115 +429,130 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
       </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
       </c>
       <c r="F3" t="s">
         <v>12</v>
       </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>
       </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>12</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D3" r:id="rId2"/>
-    <hyperlink ref="D4" r:id="rId3"/>
-    <hyperlink ref="D5" r:id="rId4"/>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add test data reader
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1266D14A-0A66-4FE2-BA68-3591730FFF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateUserCredentials" sheetId="1" r:id="rId1"/>
+    <sheet name="All Leave" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Role</t>
   </si>
@@ -59,12 +61,27 @@
   </si>
   <si>
     <t>Employee_123</t>
+  </si>
+  <si>
+    <t>EmployeeName</t>
+  </si>
+  <si>
+    <t>LeaveType</t>
+  </si>
+  <si>
+    <t>Entitlement</t>
+  </si>
+  <si>
+    <t>Ravi M B</t>
+  </si>
+  <si>
+    <t>CAN - Personal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -94,8 +111,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -114,9 +134,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -154,9 +174,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -191,7 +211,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -226,7 +246,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -399,11 +419,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -423,7 +443,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -443,7 +463,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -461,6 +481,51 @@
       </c>
       <c r="F3" t="s">
         <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2CE7DB5-7FD9-4C48-A615-A43DFAB39DE2}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>100001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rohini: Create User Credentials - Duplicate Username Handled
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
   <si>
     <t>Role</t>
   </si>
@@ -59,6 +59,15 @@
   </si>
   <si>
     <t>Employee@123</t>
+  </si>
+  <si>
+    <t>Admin 1</t>
+  </si>
+  <si>
+    <t>Employee 1</t>
+  </si>
+  <si>
+    <t>DuplicateUser</t>
   </si>
 </sst>
 </file>
@@ -445,7 +454,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -468,7 +477,7 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -484,7 +493,27 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E4" s="1"/>
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E5" s="1"/>
@@ -493,7 +522,9 @@
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rohini: Create User Credentials - Mismatch password, Empty validation
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
   <si>
     <t>Role</t>
   </si>
@@ -68,6 +68,15 @@
   </si>
   <si>
     <t>DuplicateUser</t>
+  </si>
+  <si>
+    <t>WithoutMandatoryField</t>
+  </si>
+  <si>
+    <t>PasswordMismatch</t>
+  </si>
+  <si>
+    <t>Admin1234</t>
   </si>
 </sst>
 </file>
@@ -420,8 +429,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="38.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -516,15 +528,45 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
       <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
     <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E6" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
attendance and buzz tests
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD9FF82-C5C9-4539-B265-2A7A99425493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateUserCredentials" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateUser" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
   <si>
     <t>Role</t>
   </si>
@@ -68,12 +70,33 @@
   </si>
   <si>
     <t>DuplicateUser</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>empid</t>
+  </si>
+  <si>
+    <t>ScriptX_Admin</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>ScriptX_Employee</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -134,9 +157,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -174,9 +197,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -211,7 +234,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -246,7 +269,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -419,11 +442,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -446,7 +469,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -469,7 +492,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -492,7 +515,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -515,16 +538,62 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D7F426-6B88-4E29-9DB5-39F4E9DC39CF}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3">
+        <v>555</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added employee buzz module
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72DAA1E-ED69-4E4B-8829-5F3D01C8E6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateUserCredentials" sheetId="1" r:id="rId1"/>
+    <sheet name="BuzzDetails" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t>Role</t>
   </si>
@@ -68,12 +70,24 @@
   </si>
   <si>
     <t>DuplicateUser</t>
+  </si>
+  <si>
+    <t>New Post text</t>
+  </si>
+  <si>
+    <t>Edit Post Text</t>
+  </si>
+  <si>
+    <t>I'm Happy</t>
+  </si>
+  <si>
+    <t>Today, I'm attending a party to celebrate our project's success.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -134,9 +148,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -174,9 +188,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -211,7 +225,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -246,7 +260,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -419,11 +433,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -446,7 +460,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -469,7 +483,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -492,7 +506,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -515,16 +529,46 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E5" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3189F70-F90A-41EE-934D-69BBEDB382F3}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.88671875" customWidth="1"/>
+    <col min="2" max="2" width="51.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added a new Scenario
</commit_message>
<xml_diff>
--- a/ScriptX_OrangeHRM/Configurations/TestData.xlsx
+++ b/ScriptX_OrangeHRM/Configurations/TestData.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F17996C-A305-468D-9DB6-F298ADEEEE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6651A40-952E-4ED8-9645-56F52A39E2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateUserCredentials" sheetId="1" r:id="rId1"/>
@@ -13,13 +13,14 @@
     <sheet name="CreateUser" sheetId="3" r:id="rId3"/>
     <sheet name="ContactDetails" sheetId="5" r:id="rId4"/>
     <sheet name="EmergencyContact" sheetId="6" r:id="rId5"/>
+    <sheet name="SalaryDetails" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="61">
   <si>
     <t>Role</t>
   </si>
@@ -169,6 +170,39 @@
   </si>
   <si>
     <t>044-12345678</t>
+  </si>
+  <si>
+    <t>salary_component</t>
+  </si>
+  <si>
+    <t>pay_grade</t>
+  </si>
+  <si>
+    <t>pay_frequency</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>Basic Salary</t>
+  </si>
+  <si>
+    <t>Grade 1</t>
+  </si>
+  <si>
+    <t>Monthly</t>
+  </si>
+  <si>
+    <t>Indian Rupee - INR</t>
+  </si>
+  <si>
+    <t>Monthly CTC</t>
   </si>
 </sst>
 </file>
@@ -886,4 +920,62 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7D3B135-8F78-4C54-A551-0CFE180E859C}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" customWidth="1"/>
+    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" customWidth="1"/>
+    <col min="6" max="6" width="29.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="5">
+        <v>50000</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>